<commit_message>
update eoi with excel
</commit_message>
<xml_diff>
--- a/data/opportunities.xlsx
+++ b/data/opportunities.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Opportunities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -540,33 +540,108 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Industry Collaboration Opportunity - NSRC</t>
+          <t>Fw: EOI Request – Industry Collaboration Opportunity with Office of Developmental Affairs (Presidential Court)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Opportunity</t>
+          <t>Call for Interest</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>16/03/26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>National Search and Rescue Centre (NSRC)</t>
+          <t>Office of Developmental Affairs (Presidential Court)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>partnerships@mbzuai.ac.ae</t>
+          <t>Ilham.Saeed@mbzuai.ac.ae</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>• scale development programs.
+• Strategic program design
+• Cross-entity coordination
+• Monitoring and evaluation of development initiatives
+• Supporting UAE leadership humanitarian vision
+• More details found in documents attached
+• enabled institutional knowledge and analytics platform for the Social Affairs Sector that transforms flagship books, internal publications, policy documents and research outputs into:
+• A structured, authoritative digital knowledge base
+• An AI-powered exploration, summarization and insight-generation system
+• An executive analytical and reporting environment</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mbzuai.ac.ae/</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>________________________________
+From: Ilham Saeed &lt;Ilham.Saeed@mbzuai.ac.ae&gt;
+Sent: Monday, 9 March 2026 12:42 PM
+Cc: Ramzi Ben Ouaghrem &lt;Ramzi.BenOuaghrem@mbzuai.ac.ae&gt;; Sultan Al Hajji &lt;Sultan.Alhajji@mbzuai.ac.ae&gt;
+Subject: EOI Request – Industry Collaboration Opportunity with Office of Developmental Affairs (Presidential Court)
+Dear Department Chairs,
+We are reaching out to request expressions of interest for a new industry collaboration opportunity. Kindly share this with your depart</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>innovation</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Industry Collaboration Opportunity - NSRC</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>National Search and Rescue Centre (NSRC)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>partnerships@mbzuai.ac.ae</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>• Intelligent Signal Processing
 • Automated Datum Estimation and Environmental Data Fusion
@@ -577,8 +652,8 @@
 • Trustworthy and Safety-Critical AI</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Dear Department Chairs,
 We are reaching out to request expressions of interest for a new industry collaboration opportunity. Kindly share this with your department and/or refer it to the most suitable faculty member.
@@ -587,24 +662,24 @@
 The National Search and Rescue Centre (NSRC) is the UAE's central federal agency responsible for planning, coordinating, and executing all national search and rescue (SAR) operations across land, sea, an</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>new</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>innovation</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N2"/>
+  <autoFilter ref="A1:N3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>